<commit_message>
updated procurement data driven
</commit_message>
<xml_diff>
--- a/Oracle_Tool_Automation/data/Oracle_TestData.xlsx
+++ b/Oracle_Tool_Automation/data/Oracle_TestData.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Oracle Fusion Workspace\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PhaniKumarMaddi\git\OracleRepository\Oracle_Tool_Automation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21001236-CFBA-4787-9A95-1A4690E2404C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6C7259-3A03-43BF-86AB-913204BC06D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7F354CF8-B21A-407D-B732-A31BC19C7C54}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{7F354CF8-B21A-407D-B732-A31BC19C7C54}"/>
   </bookViews>
   <sheets>
     <sheet name="Procurement" sheetId="1" r:id="rId1"/>
+    <sheet name="Procuremen_WithoutRequisition" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>Item Description</t>
   </si>
@@ -58,6 +59,45 @@
   </si>
   <si>
     <t>Each</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>CRITICAL RIVER LOCATION</t>
+  </si>
+  <si>
+    <t>Ship to</t>
+  </si>
+  <si>
+    <t>Item in PO</t>
+  </si>
+  <si>
+    <t>CR1002</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>04</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>2026</t>
   </si>
 </sst>
 </file>
@@ -127,11 +167,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -480,14 +523,68 @@
       <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1">
-        <v>3</v>
+      <c r="C2" s="4" t="s">
+        <v>8</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="1">
-        <v>30</v>
+      <c r="E2" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A33F0F74-BC08-44D3-96F2-D90553CCF308}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="26.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>